<commit_message>
Tdu update api 1.6 and backoffice (#1)
- Update backend, shared clients and backoffice for API 1.6 with the correct routes.
- Synchronize schemas, API helpers and hooks across the three layers.
- Update backend/shared tests and expand admin-interface coverage.
- Correct errors in backoffice screens.
</commit_message>
<xml_diff>
--- a/backend/data/excel_structure_guide.xlsx
+++ b/backend/data/excel_structure_guide.xlsx
@@ -425,14 +425,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="52" customWidth="1" min="2" max="2"/>
-    <col width="73" customWidth="1" min="3" max="3"/>
+    <col width="54" customWidth="1" min="2" max="2"/>
+    <col width="77" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="71" customWidth="1" min="5" max="5"/>
+    <col width="80" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -678,6 +678,60 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>content_lists</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Flexible content organization lists (NEW in API 1.6)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>title (required), thumbnail_format (required), content_items, content_types</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>_ref_name</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Can mix programs, seasons, and media descriptions. thumbnail_format must be: small_square, medium_portrait, large_landscape, or vertical_mobile</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>screen_contents</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Complete screen layout management (NEW in API 1.6)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>title (required), content_lists, screen_type</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>_ref_name</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Organizes content lists into screen layouts. References content_lists by name.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>